<commit_message>
the-hotel-gurus: deck + workbook rebuilt with retitled articles
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/the-hotel-gurus/keyword-research.xlsx
+++ b/decks/the-hotel-gurus/keyword-research.xlsx
@@ -791,7 +791,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Group Business Solutions for Hotel Blocks: What Exists Beyond DIY</t>
+          <t>Group Hotel Block Services: What Exists Beyond Doing It Yourself</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>How to Negotiate Group Hotel Rates for a Conference</t>
+          <t>Conference Hotel Rates: The Negotiation Playbook for Event Planners</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>How to Book Hotel Rooms for a Group, Step by Step</t>
+          <t>How to Book Hotel Rooms for a Group: With or Without a Room Block</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Can You Request Special Rates for Wedding Guests?</t>
+          <t>How to Ask a Hotel for Special Wedding Guest Rates (Wording Included)</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>Group vs. Individual Hotel Rates: The Difference, Explained</t>
+          <t>Group vs. Individual Hotel Rates: How the Pricing Actually Works</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">

</xml_diff>